<commit_message>
addded a simple serial parser
</commit_message>
<xml_diff>
--- a/docs/HX3_FPGA_SPI.xlsx
+++ b/docs/HX3_FPGA_SPI.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="360" yWindow="60" windowWidth="30915" windowHeight="16425" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="60" windowWidth="30915" windowHeight="16425"/>
   </bookViews>
   <sheets>
     <sheet name="FPGA SPI" sheetId="3" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="347">
   <si>
     <t>Name</t>
   </si>
@@ -847,97 +847,220 @@
     <t>AO28 LOUDN BASS</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_SystemInits</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = 496;</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_VibKnobMode</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 1; // #1497</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_RestoreCommonPresetMask</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 2; // #1498</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_ButtonMask0</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 3; // #1499 ALT</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_ButtonMask1</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 4; // #1500 ALT</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_ConfBits1</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 5; // #1501</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_ConfBits2</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 6; // #1502</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_ADCconfig</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 7; // #1503</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_1stDBselect</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 8; // #1504</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_2ndDBselect</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 9; // #1505</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_PedalDBsetup</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 10; // #1506</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_ADCscaling</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 11; // #1507</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_DeviceType</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 13; // #1509</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_PresetStructure</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 14; // #1510</t>
   </si>
   <si>
-    <t xml:space="preserve">  c_EditMagicFlagIdx</t>
-  </si>
-  <si>
     <t xml:space="preserve"> Word = c_SystemInits + 15; // #1511</t>
   </si>
   <si>
     <t>C++# defines</t>
+  </si>
+  <si>
+    <t>c_SystemInits</t>
+  </si>
+  <si>
+    <t>c_VibKnobMode</t>
+  </si>
+  <si>
+    <t>c_RestoreCommonPresetMask</t>
+  </si>
+  <si>
+    <t>c_ButtonMask0</t>
+  </si>
+  <si>
+    <t>c_ButtonMask1</t>
+  </si>
+  <si>
+    <t>c_ConfBits1</t>
+  </si>
+  <si>
+    <t>c_ConfBits2</t>
+  </si>
+  <si>
+    <t>c_ADCconfig</t>
+  </si>
+  <si>
+    <t>c_1stDBselect</t>
+  </si>
+  <si>
+    <t>c_2ndDBselect</t>
+  </si>
+  <si>
+    <t>c_PedalDBsetup</t>
+  </si>
+  <si>
+    <t>c_ADCscaling</t>
+  </si>
+  <si>
+    <t>c_DeviceType</t>
+  </si>
+  <si>
+    <t>c_PresetStructure</t>
+  </si>
+  <si>
+    <t>c_EditMagicFlagIdx</t>
+  </si>
+  <si>
+    <t>phases 0</t>
+  </si>
+  <si>
+    <t>phases 1</t>
+  </si>
+  <si>
+    <t>phases 2</t>
+  </si>
+  <si>
+    <t>phases 3</t>
+  </si>
+  <si>
+    <t>phases 4</t>
+  </si>
+  <si>
+    <t>phases 5</t>
+  </si>
+  <si>
+    <t>phases 6</t>
+  </si>
+  <si>
+    <t>phases 7</t>
+  </si>
+  <si>
+    <t>phases 8</t>
+  </si>
+  <si>
+    <t>phases 9</t>
+  </si>
+  <si>
+    <t>phases 10</t>
+  </si>
+  <si>
+    <t>phases 11</t>
+  </si>
+  <si>
+    <t>inits 0</t>
+  </si>
+  <si>
+    <t>inits 1</t>
+  </si>
+  <si>
+    <t>inits 2</t>
+  </si>
+  <si>
+    <t>inits 3</t>
+  </si>
+  <si>
+    <t>inits 4</t>
+  </si>
+  <si>
+    <t>inits 5</t>
+  </si>
+  <si>
+    <t>inits 6</t>
+  </si>
+  <si>
+    <t>inits 7</t>
+  </si>
+  <si>
+    <t>inits 8</t>
+  </si>
+  <si>
+    <t>inits 9</t>
+  </si>
+  <si>
+    <t>inits 10</t>
+  </si>
+  <si>
+    <t>inits 11</t>
+  </si>
+  <si>
+    <t>inits 12</t>
+  </si>
+  <si>
+    <t>inits 13</t>
+  </si>
+  <si>
+    <t>inits 14</t>
+  </si>
+  <si>
+    <t>inits 15</t>
+  </si>
+  <si>
+    <t>inits 16</t>
+  </si>
+  <si>
+    <t>inits 17</t>
+  </si>
+  <si>
+    <t>inits 18</t>
+  </si>
+  <si>
+    <t>inits 19</t>
+  </si>
+  <si>
+    <t>inits 20</t>
+  </si>
+  <si>
+    <t>inits 21</t>
+  </si>
+  <si>
+    <t>inits 22</t>
+  </si>
+  <si>
+    <t>inits 23</t>
+  </si>
+  <si>
+    <t>inits 24</t>
+  </si>
+  <si>
+    <t>inits 25</t>
+  </si>
+  <si>
+    <t>inits 26</t>
+  </si>
+  <si>
+    <t>inits 27</t>
+  </si>
+  <si>
+    <t>inits 28</t>
   </si>
 </sst>
 </file>
@@ -1011,7 +1134,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1072,6 +1195,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1085,7 +1214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1163,6 +1292,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1474,7 +1606,7 @@
   <cols>
     <col min="1" max="1" width="8.42578125" style="3" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" style="5" customWidth="1"/>
-    <col min="3" max="3" width="23.140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="33.42578125" style="5" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" style="5"/>
     <col min="5" max="5" width="36" style="5" customWidth="1"/>
     <col min="6" max="6" width="32.28515625" style="5" customWidth="1"/>
@@ -4369,7 +4501,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_3 = 163;</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A113" s="3">
         <v>164</v>
       </c>
@@ -4388,7 +4520,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_4 = 164;</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A114" s="3">
         <v>165</v>
       </c>
@@ -4407,7 +4539,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_5 = 165;</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A115" s="3">
         <v>166</v>
       </c>
@@ -4426,7 +4558,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_6 = 166;</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A116" s="3">
         <v>167</v>
       </c>
@@ -4445,7 +4577,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_7 = 167;</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A117" s="3">
         <v>168</v>
       </c>
@@ -4464,7 +4596,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_8 = 168;</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A118" s="3">
         <v>169</v>
       </c>
@@ -4483,7 +4615,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_9 = 169;</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A119" s="3">
         <v>170</v>
       </c>
@@ -4502,7 +4634,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_10 = 170;</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A120" s="3">
         <v>171</v>
       </c>
@@ -4521,7 +4653,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_11 = 171;</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A121" s="3">
         <v>172</v>
       </c>
@@ -4540,7 +4672,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_12 = 172;</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A122" s="3">
         <v>173</v>
       </c>
@@ -4559,7 +4691,7 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_13 = 173;</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A123" s="3">
         <v>174</v>
       </c>
@@ -4578,13 +4710,13 @@
         <v xml:space="preserve">  c_spi_lc_line_dly_14 = 174;</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A124" s="3">
         <v>175</v>
       </c>
       <c r="F124" s="21"/>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A125" s="3">
         <v>176</v>
       </c>
@@ -4599,8 +4731,11 @@
       <c r="G125" s="5" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I125" s="5" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A126" s="3">
         <v>177</v>
       </c>
@@ -4618,8 +4753,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_speed_horn = 177;</v>
       </c>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I126" s="5" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A127" s="3">
         <v>178</v>
       </c>
@@ -4637,8 +4775,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_speed_rotor = 178;</v>
       </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I127" s="5" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A128" s="3">
         <v>179</v>
       </c>
@@ -4659,8 +4800,11 @@
       <c r="G128" s="5" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I128" s="5" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A129" s="3">
         <v>180</v>
       </c>
@@ -4678,8 +4822,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_inp_lvl = 180;</v>
       </c>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I129" s="5" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A130" s="3">
         <v>181</v>
       </c>
@@ -4697,8 +4844,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_horn_lvl = 181;</v>
       </c>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I130" s="5" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A131" s="3">
         <v>182</v>
       </c>
@@ -4716,8 +4866,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_rotor_lvl = 182;</v>
       </c>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I131" s="5" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A132" s="3">
         <v>183</v>
       </c>
@@ -4735,8 +4888,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_horn_near_refl_lvl = 183;</v>
       </c>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I132" s="5" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A133" s="3">
         <v>184</v>
       </c>
@@ -4754,8 +4910,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_horn_room_refl_lvl = 184;</v>
       </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I133" s="5" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A134" s="3">
         <v>185</v>
       </c>
@@ -4773,8 +4932,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_xover_frequ = 185;</v>
       </c>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I134" s="5" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A135" s="3">
         <v>186</v>
       </c>
@@ -4786,8 +4948,11 @@
       </c>
       <c r="E135" s="17"/>
       <c r="F135" s="21"/>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I135" s="5" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A136" s="3">
         <v>187</v>
       </c>
@@ -4805,8 +4970,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_pre_dly = 187;</v>
       </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I136" s="5" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A137" s="3">
         <v>188</v>
       </c>
@@ -4824,8 +4992,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_diffuse_1 = 188;</v>
       </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I137" s="5" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A138" s="3">
         <v>189</v>
       </c>
@@ -4843,8 +5014,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_diffuse_2 = 189;</v>
       </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I138" s="5" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A139" s="3">
         <v>190</v>
       </c>
@@ -4862,8 +5036,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_diffuse_3 = 190;</v>
       </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I139" s="5" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A140" s="3">
         <v>191</v>
       </c>
@@ -4881,8 +5058,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_rotry_diffuse_4 = 191;</v>
       </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I140" s="5" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A141" s="3">
         <v>192</v>
       </c>
@@ -4903,8 +5083,11 @@
       <c r="G141" s="5" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I141" s="5" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A142" s="3">
         <v>193</v>
       </c>
@@ -4922,8 +5105,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_main_r = 193;</v>
       </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I142" s="5" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A143" s="3">
         <v>194</v>
       </c>
@@ -4941,8 +5127,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_refl_1_l_near = 194;</v>
       </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I143" s="5" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A144" s="3">
         <v>195</v>
       </c>
@@ -4960,8 +5149,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_refl_1_r_near = 195;</v>
       </c>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I144" s="5" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A145" s="3">
         <v>196</v>
       </c>
@@ -4979,8 +5171,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_refl_2_l_far = 196;</v>
       </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I145" s="5" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A146" s="3">
         <v>197</v>
       </c>
@@ -4998,8 +5193,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_refl_2_r_far = 197;</v>
       </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I146" s="5" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A147" s="3">
         <v>198</v>
       </c>
@@ -5017,8 +5215,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_throb_l = 198;</v>
       </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I147" s="5" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A148" s="3">
         <v>199</v>
       </c>
@@ -5036,8 +5237,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_throb_r = 199;</v>
       </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I148" s="5" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A149" s="3">
         <v>200</v>
       </c>
@@ -5055,8 +5259,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_cab = 200;</v>
       </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I149" s="5" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A150" s="3">
         <v>201</v>
       </c>
@@ -5074,8 +5281,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_rotor_main = 201;</v>
       </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I150" s="5" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A151" s="3">
         <v>202</v>
       </c>
@@ -5093,8 +5303,11 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_rotor_refl = 202;</v>
       </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I151" s="5" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A152" s="3">
         <v>203</v>
       </c>
@@ -5113,8 +5326,11 @@
         <v xml:space="preserve">  c_spi_lfo_mod_rotor_throb = 203;</v>
       </c>
       <c r="G152" s="10"/>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I152" s="5" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A153" s="3">
         <v>204</v>
       </c>
@@ -5135,32 +5351,35 @@
       <c r="G153" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I153" s="5" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A154" s="3">
         <v>205</v>
       </c>
       <c r="F154" s="21"/>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
       <c r="F155" s="21"/>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
       <c r="F156" s="21"/>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A157" s="3">
         <v>222</v>
       </c>
       <c r="F157" s="21"/>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A158" s="3">
         <v>223</v>
       </c>
       <c r="F158" s="21"/>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A159" s="3">
         <v>224</v>
       </c>
@@ -5181,8 +5400,11 @@
       <c r="G159" s="5" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I159" s="5" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A160" s="3">
         <v>225</v>
       </c>
@@ -5200,8 +5422,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_main_r = 225;</v>
       </c>
-    </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I160" s="27" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A161" s="3">
         <v>226</v>
       </c>
@@ -5219,8 +5444,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_refl_1_l_near_cab = 226;</v>
       </c>
-    </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I161" s="5" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A162" s="3">
         <v>227</v>
       </c>
@@ -5238,8 +5466,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_refl_1_r_near_cab = 227;</v>
       </c>
-    </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I162" s="27" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A163" s="3">
         <v>228</v>
       </c>
@@ -5257,8 +5488,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_refl_2_l__far = 228;</v>
       </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I163" s="5" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A164" s="3">
         <v>229</v>
       </c>
@@ -5276,8 +5510,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_refl_2_r_far = 229;</v>
       </c>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I164" s="27" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A165" s="3">
         <v>230</v>
       </c>
@@ -5295,8 +5532,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_throb_l__2_khz = 230;</v>
       </c>
-    </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I165" s="5" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A166" s="3">
         <v>231</v>
       </c>
@@ -5314,8 +5554,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_throb_r_2_khz = 231;</v>
       </c>
-    </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I166" s="27" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A167" s="3">
         <v>232</v>
       </c>
@@ -5333,8 +5576,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_horn_cab_4x = 232;</v>
       </c>
-    </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I167" s="5" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A168" s="3">
         <v>233</v>
       </c>
@@ -5352,8 +5598,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_rotor_main = 233;</v>
       </c>
-    </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I168" s="5" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A169" s="3">
         <v>234</v>
       </c>
@@ -5371,8 +5620,11 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_rotor_refl = 234;</v>
       </c>
-    </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I169" s="5" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A170" s="3">
         <v>235</v>
       </c>
@@ -5390,28 +5642,31 @@
         <f t="shared" si="18"/>
         <v xml:space="preserve">  c_spi_lfo_phase_offset_rotor_throb = 235;</v>
       </c>
-    </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I170" s="5" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A171" s="3">
         <v>236</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A172" s="3">
         <v>237</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A173" s="3">
         <v>238</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A174" s="3">
         <v>239</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A175" s="3">
         <v>240</v>
       </c>
@@ -5436,7 +5691,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A176" s="3">
         <v>241</v>
       </c>
@@ -5584,7 +5839,7 @@
         <v>164</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>305</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -5592,14 +5847,18 @@
         <v>496</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>275</v>
+        <v>291</v>
       </c>
       <c r="D2" s="26" t="str">
         <f>UPPER(SUBSTITUTE(B2,"c_","OFS_"))</f>
-        <v xml:space="preserve">  OFS_SYSTEMINITS</v>
+        <v>OFS_SYSTEMINITS</v>
+      </c>
+      <c r="E2" s="26" t="str">
+        <f>CONCATENATE("#define ",D2," ",A2)</f>
+        <v>#define OFS_SYSTEMINITS 496</v>
       </c>
       <c r="H2" s="26" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5607,14 +5866,18 @@
         <v>497</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>277</v>
+        <v>292</v>
       </c>
       <c r="D3" s="26" t="str">
         <f t="shared" ref="D3:D17" si="0">UPPER(SUBSTITUTE(B3,"c_","OFS_"))</f>
-        <v xml:space="preserve">  OFS_VIBKNOBMODE</v>
+        <v>OFS_VIBKNOBMODE</v>
+      </c>
+      <c r="E3" s="26" t="str">
+        <f t="shared" ref="E3:E17" si="1">CONCATENATE("#define ",D3," ",A3)</f>
+        <v>#define OFS_VIBKNOBMODE 497</v>
       </c>
       <c r="H3" s="26" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5622,14 +5885,18 @@
         <v>498</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>279</v>
+        <v>293</v>
       </c>
       <c r="D4" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_RESTORECOMMONPRESETMASK</v>
+        <v>OFS_RESTORECOMMONPRESETMASK</v>
+      </c>
+      <c r="E4" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_RESTORECOMMONPRESETMASK 498</v>
       </c>
       <c r="H4" s="26" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5637,14 +5904,18 @@
         <v>499</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>281</v>
+        <v>294</v>
       </c>
       <c r="D5" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_BUTTONMASK0</v>
+        <v>OFS_BUTTONMASK0</v>
+      </c>
+      <c r="E5" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_BUTTONMASK0 499</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
@@ -5652,14 +5923,18 @@
         <v>500</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="D6" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_BUTTONMASK1</v>
+        <v>OFS_BUTTONMASK1</v>
+      </c>
+      <c r="E6" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_BUTTONMASK1 500</v>
       </c>
       <c r="H6" s="26" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
@@ -5667,14 +5942,18 @@
         <v>501</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>285</v>
+        <v>296</v>
       </c>
       <c r="D7" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_CONFBITS1</v>
+        <v>OFS_CONFBITS1</v>
+      </c>
+      <c r="E7" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_CONFBITS1 501</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5682,14 +5961,18 @@
         <v>502</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>287</v>
+        <v>297</v>
       </c>
       <c r="D8" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_CONFBITS2</v>
+        <v>OFS_CONFBITS2</v>
+      </c>
+      <c r="E8" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_CONFBITS2 502</v>
       </c>
       <c r="H8" s="26" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5697,14 +5980,18 @@
         <v>503</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="D9" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_ADCCONFIG</v>
+        <v>OFS_ADCCONFIG</v>
+      </c>
+      <c r="E9" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_ADCCONFIG 503</v>
       </c>
       <c r="H9" s="26" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5712,14 +5999,18 @@
         <v>504</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="D10" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_1STDBSELECT</v>
+        <v>OFS_1STDBSELECT</v>
+      </c>
+      <c r="E10" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_1STDBSELECT 504</v>
       </c>
       <c r="H10" s="26" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
@@ -5727,14 +6018,18 @@
         <v>505</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="D11" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_2NDDBSELECT</v>
+        <v>OFS_2NDDBSELECT</v>
+      </c>
+      <c r="E11" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_2NDDBSELECT 505</v>
       </c>
       <c r="H11" s="26" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -5742,14 +6037,18 @@
         <v>506</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="D12" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_PEDALDBSETUP</v>
+        <v>OFS_PEDALDBSETUP</v>
+      </c>
+      <c r="E12" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_PEDALDBSETUP 506</v>
       </c>
       <c r="H12" s="26" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -5757,14 +6056,18 @@
         <v>507</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="D13" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_ADCSCALING</v>
+        <v>OFS_ADCSCALING</v>
+      </c>
+      <c r="E13" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_ADCSCALING 507</v>
       </c>
       <c r="H13" s="26" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -5781,14 +6084,18 @@
         <v>509</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="D15" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_DEVICETYPE</v>
+        <v>OFS_DEVICETYPE</v>
+      </c>
+      <c r="E15" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_DEVICETYPE 509</v>
       </c>
       <c r="H15" s="26" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
@@ -5796,14 +6103,18 @@
         <v>510</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D16" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_PRESETSTRUCTURE</v>
+        <v>OFS_PRESETSTRUCTURE</v>
+      </c>
+      <c r="E16" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_PRESETSTRUCTURE 510</v>
       </c>
       <c r="H16" s="26" t="s">
-        <v>302</v>
+        <v>288</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -5811,17 +6122,22 @@
         <v>511</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D17" s="26" t="str">
         <f t="shared" si="0"/>
-        <v xml:space="preserve">  OFS_EDITMAGICFLAGIDX</v>
+        <v>OFS_EDITMAGICFLAGIDX</v>
+      </c>
+      <c r="E17" s="26" t="str">
+        <f t="shared" si="1"/>
+        <v>#define OFS_EDITMAGICFLAGIDX 511</v>
       </c>
       <c r="H17" s="26" t="s">
-        <v>304</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new menupanell and panel16
</commit_message>
<xml_diff>
--- a/docs/HX3_FPGA_SPI.xlsx
+++ b/docs/HX3_FPGA_SPI.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="347">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="348">
   <si>
     <t>Name</t>
   </si>
@@ -1061,6 +1061,9 @@
   </si>
   <si>
     <t>inits 28</t>
+  </si>
+  <si>
+    <t>in liveCtrl berechnet</t>
   </si>
 </sst>
 </file>
@@ -4804,7 +4807,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A129" s="3">
         <v>180</v>
       </c>
@@ -4826,7 +4829,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A130" s="3">
         <v>181</v>
       </c>
@@ -4848,7 +4851,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A131" s="3">
         <v>182</v>
       </c>
@@ -4870,7 +4873,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A132" s="3">
         <v>183</v>
       </c>
@@ -4892,7 +4895,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A133" s="3">
         <v>184</v>
       </c>
@@ -4914,7 +4917,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A134" s="3">
         <v>185</v>
       </c>
@@ -4936,7 +4939,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A135" s="3">
         <v>186</v>
       </c>
@@ -4952,7 +4955,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A136" s="3">
         <v>187</v>
       </c>
@@ -4974,7 +4977,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A137" s="3">
         <v>188</v>
       </c>
@@ -4996,7 +4999,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A138" s="3">
         <v>189</v>
       </c>
@@ -5018,7 +5021,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A139" s="3">
         <v>190</v>
       </c>
@@ -5040,7 +5043,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A140" s="3">
         <v>191</v>
       </c>
@@ -5062,7 +5065,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A141" s="3">
         <v>192</v>
       </c>
@@ -5087,7 +5090,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A142" s="3">
         <v>193</v>
       </c>
@@ -5105,11 +5108,14 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_main_r = 193;</v>
       </c>
-      <c r="I142" s="5" t="s">
+      <c r="I142" s="27" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J142" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A143" s="3">
         <v>194</v>
       </c>
@@ -5131,7 +5137,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A144" s="3">
         <v>195</v>
       </c>
@@ -5149,11 +5155,14 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_refl_1_r_near = 195;</v>
       </c>
-      <c r="I144" s="5" t="s">
+      <c r="I144" s="27" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J144" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A145" s="3">
         <v>196</v>
       </c>
@@ -5175,7 +5184,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A146" s="3">
         <v>197</v>
       </c>
@@ -5193,11 +5202,14 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_refl_2_r_far = 197;</v>
       </c>
-      <c r="I146" s="5" t="s">
+      <c r="I146" s="27" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J146" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A147" s="3">
         <v>198</v>
       </c>
@@ -5219,7 +5231,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A148" s="3">
         <v>199</v>
       </c>
@@ -5237,11 +5249,14 @@
         <f t="shared" si="15"/>
         <v xml:space="preserve">  c_spi_lfo_mod_horn_throb_r = 199;</v>
       </c>
-      <c r="I148" s="5" t="s">
+      <c r="I148" s="27" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J148" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A149" s="3">
         <v>200</v>
       </c>
@@ -5263,7 +5278,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A150" s="3">
         <v>201</v>
       </c>
@@ -5285,7 +5300,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A151" s="3">
         <v>202</v>
       </c>
@@ -5307,7 +5322,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A152" s="3">
         <v>203</v>
       </c>
@@ -5330,7 +5345,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A153" s="3">
         <v>204</v>
       </c>
@@ -5355,31 +5370,31 @@
         <v>346</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A154" s="3">
         <v>205</v>
       </c>
       <c r="F154" s="21"/>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F155" s="21"/>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
       <c r="F156" s="21"/>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A157" s="3">
         <v>222</v>
       </c>
       <c r="F157" s="21"/>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A158" s="3">
         <v>223</v>
       </c>
       <c r="F158" s="21"/>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A159" s="3">
         <v>224</v>
       </c>
@@ -5404,7 +5419,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A160" s="3">
         <v>225</v>
       </c>
@@ -5425,8 +5440,11 @@
       <c r="I160" s="27" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J160" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A161" s="3">
         <v>226</v>
       </c>
@@ -5448,7 +5466,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A162" s="3">
         <v>227</v>
       </c>
@@ -5469,8 +5487,11 @@
       <c r="I162" s="27" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J162" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A163" s="3">
         <v>228</v>
       </c>
@@ -5492,7 +5513,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A164" s="3">
         <v>229</v>
       </c>
@@ -5513,8 +5534,11 @@
       <c r="I164" s="27" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J164" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A165" s="3">
         <v>230</v>
       </c>
@@ -5536,7 +5560,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A166" s="3">
         <v>231</v>
       </c>
@@ -5557,8 +5581,11 @@
       <c r="I166" s="27" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J166" s="5" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A167" s="3">
         <v>232</v>
       </c>
@@ -5580,7 +5607,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A168" s="3">
         <v>233</v>
       </c>
@@ -5602,7 +5629,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A169" s="3">
         <v>234</v>
       </c>
@@ -5624,7 +5651,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A170" s="3">
         <v>235</v>
       </c>
@@ -5646,27 +5673,27 @@
         <v>317</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A171" s="3">
         <v>236</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A172" s="3">
         <v>237</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A173" s="3">
         <v>238</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A174" s="3">
         <v>239</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A175" s="3">
         <v>240</v>
       </c>
@@ -5691,7 +5718,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A176" s="3">
         <v>241</v>
       </c>

</xml_diff>